<commit_message>
docs: add course taxonomy framework
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R6ddfd87f6e8b4ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R067a483078e049e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="R8fa6f856eed34f5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="Rb0ccd2f4546f42d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R0654be7296e44b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Re1b2a8c05d6e4417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R54a82894b0ea4883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R1d696d814609460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="Rad33e9594d444e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R199c2dd66a6d4a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="R41d5016331be4372"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="Rbfb6ef1c07ee482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R7cc1e444a6f54431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Re72c2369e8484a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R9c18b21bb7d244af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="Rf55cf1da45ce4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R1848f2f70b914950"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,13 +53,34 @@
       <x:sz val="11"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF101828"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E53FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF3FF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -108,7 +130,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -178,6 +200,50 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2055,4 +2121,515 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2E53FA"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="26" t="str">
+        <x:v>课程分类体系｜开发任务、内容主题与技术栈</x:v>
+      </x:c>
+      <x:c r="B1" s="27"/>
+      <x:c r="C1" s="27"/>
+      <x:c r="D1" s="27"/>
+      <x:c r="E1" s="27"/>
+      <x:c r="F1" s="27"/>
+      <x:c r="G1" s="27"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="28" t="str">
+        <x:v>一级入口按用户开发任务组织；业务三大类作为内容主题；技术路线、框架与环境作为可多选标签。</x:v>
+      </x:c>
+      <x:c r="B2" s="27"/>
+      <x:c r="C2" s="27"/>
+      <x:c r="D2" s="27"/>
+      <x:c r="E2" s="27"/>
+      <x:c r="F2" s="27"/>
+      <x:c r="G2" s="27"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="34" t="str">
+        <x:v>1. 主要开发任务：面向用户的一级分类</x:v>
+      </x:c>
+      <x:c r="B4" s="34"/>
+      <x:c r="C4" s="34"/>
+      <x:c r="D4" s="34"/>
+      <x:c r="E4" s="34"/>
+      <x:c r="F4" s="34"/>
+      <x:c r="G4" s="34"/>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="46" t="str">
+        <x:v>主要开发任务</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>分类描述</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>建议二级任务</x:v>
+      </x:c>
+      <x:c r="D5" s="47" t="str">
+        <x:v>主要用户角色</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>典型场景</x:v>
+      </x:c>
+      <x:c r="F5" s="47" t="str">
+        <x:v>完成结果</x:v>
+      </x:c>
+      <x:c r="G5" s="48" t="str">
+        <x:v>产品使用方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="58" customHeight="1">
+      <x:c r="A6" s="49" t="str">
+        <x:v>模型训练</x:v>
+      </x:c>
+      <x:c r="B6" s="49" t="str">
+        <x:v>完成数据准备、模型构建、训练编排和单机或分布式训练。</x:v>
+      </x:c>
+      <x:c r="C6" s="49" t="str">
+        <x:v>环境与数据准备；模型构建；训练编排；分布式训练；混合精度；训练性能优化</x:v>
+      </x:c>
+      <x:c r="D6" s="49" t="str">
+        <x:v>算法工程师；模型训练工程师；AI框架开发者</x:v>
+      </x:c>
+      <x:c r="E6" s="49" t="str">
+        <x:v>训练新模型、微调已有模型、扩展到多卡训练，或解决训练吞吐与收敛问题</x:v>
+      </x:c>
+      <x:c r="F6" s="49" t="str">
+        <x:v>得到可复现、可评估的训练结果</x:v>
+      </x:c>
+      <x:c r="G6" s="49" t="str">
+        <x:v>首页场景卡；课程中心一级筛选；搜索意图标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="58" customHeight="1">
+      <x:c r="A7" s="23" t="str">
+        <x:v>推理与部署</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
+        <x:v>将训练完成的模型进行转换、适配、服务化部署和运行验证。</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>模型转换；推理适配；运行时开发；服务化部署；多卡推理；推理性能验证</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="str">
+        <x:v>推理工程师；部署工程师；平台工程师</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str">
+        <x:v>把模型迁移到昇腾、部署推理服务、验证精度与性能，或处理上线失败</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="str">
+        <x:v>得到可调用、可验证的推理服务</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str">
+        <x:v>首页场景卡；课程中心一级筛选；搜索意图标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="50" t="str">
+        <x:v>算子开发</x:v>
+      </x:c>
+      <x:c r="B8" s="50" t="str">
+        <x:v>当现有算子不支持或性能不足时，完成自定义算子的实现、验证和工程化。</x:v>
+      </x:c>
+      <x:c r="C8" s="50" t="str">
+        <x:v>编程模型；编程范式；Ascend C；Triton；CATLASS；SIMD与矩阵计算；算子工程化</x:v>
+      </x:c>
+      <x:c r="D8" s="50" t="str">
+        <x:v>算子开发工程师；AI框架工程师；性能优化工程师</x:v>
+      </x:c>
+      <x:c r="E8" s="50" t="str">
+        <x:v>模型存在不支持算子、需要融合计算、需要自定义计算逻辑或提升算子性能</x:v>
+      </x:c>
+      <x:c r="F8" s="50" t="str">
+        <x:v>得到可编译、可运行、可验证的自定义算子</x:v>
+      </x:c>
+      <x:c r="G8" s="50" t="str">
+        <x:v>首页场景卡；课程中心一级筛选；搜索意图标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="23" t="str">
+        <x:v>调试与性能优化</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
+        <x:v>定位训练、推理、部署和算子开发中的功能、精度、内存、通信与性能问题。</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str">
+        <x:v>功能调试；精度问题；OOM与溢出；通信超时；性能分析；CPU/NPU孪生调试；系统调优</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="str">
+        <x:v>性能工程师；算法工程师；算子开发工程师；运维与平台工程师</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str">
+        <x:v>训练或推理报错、精度异常、OOM、通信超时、吞吐或时延未达到目标</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="str">
+        <x:v>定位根因并形成可验证的优化结果</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str">
+        <x:v>贯穿训练、推理与算子路径；可保留独立问题入口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="50" t="str">
+        <x:v>AI应用与智能体</x:v>
+      </x:c>
+      <x:c r="B10" s="50" t="str">
+        <x:v>基于大模型能力开发、评估并部署RAG、智能体和生成式AI应用。</x:v>
+      </x:c>
+      <x:c r="C10" s="50" t="str">
+        <x:v>模型接入；Prompt；RAG；工具调用；智能体编排；应用评估；服务部署</x:v>
+      </x:c>
+      <x:c r="D10" s="50" t="str">
+        <x:v>AI应用开发者；后端工程师；解决方案架构师</x:v>
+      </x:c>
+      <x:c r="E10" s="50" t="str">
+        <x:v>构建企业知识问答、智能体工作流、生成式AI服务或行业应用</x:v>
+      </x:c>
+      <x:c r="F10" s="50" t="str">
+        <x:v>得到可运行、可评估、可部署的AI应用</x:v>
+      </x:c>
+      <x:c r="G10" s="50" t="str">
+        <x:v>首页场景卡；课程中心一级筛选；搜索意图标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="34" t="str">
+        <x:v>2. 内容主题：业务三大类，作为多选标签或专题入口</x:v>
+      </x:c>
+      <x:c r="B13" s="34"/>
+      <x:c r="C13" s="34"/>
+      <x:c r="D13" s="34"/>
+      <x:c r="E13" s="34"/>
+      <x:c r="F13" s="34"/>
+    </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="A14" s="46" t="str">
+        <x:v>内容主题</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="str">
+        <x:v>主题描述</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>实际层级</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>为什么不单独作为一级任务</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>示例内容</x:v>
+      </x:c>
+      <x:c r="F14" s="48" t="str">
+        <x:v>推荐展示位置</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="49" t="str">
+        <x:v>CANN</x:v>
+      </x:c>
+      <x:c r="B15" s="49" t="str">
+        <x:v>昇腾计算软件栈、运行时、算子开发、工具链和系统能力。</x:v>
+      </x:c>
+      <x:c r="C15" s="49" t="str">
+        <x:v>底层平台与技术底座</x:v>
+      </x:c>
+      <x:c r="D15" s="49" t="str">
+        <x:v>训练、推理、部署和算子开发都会依赖CANN，无法与其他两个主题互斥</x:v>
+      </x:c>
+      <x:c r="E15" s="49" t="str">
+        <x:v>Ascend C算子开发；Triton/CATLASS；模型转换；运行时；调试调优</x:v>
+      </x:c>
+      <x:c r="F15" s="49" t="str">
+        <x:v>课程主题标签；专题页；课程中心主题筛选</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>生成式AI与大模型</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>围绕大模型训练、推理、微调、压缩和服务化的内容。</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>模型与工作负载领域</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>同一课程仍可能属于训练、推理或部署任务，并依赖CANN</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>大模型分布式训练；大模型推理；模型训推全流程</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="str">
+        <x:v>课程主题标签；专题页；课程中心主题筛选</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="50" t="str">
+        <x:v>AI应用与智能体</x:v>
+      </x:c>
+      <x:c r="B17" s="50" t="str">
+        <x:v>围绕RAG、工具调用、智能体编排及应用部署的内容。</x:v>
+      </x:c>
+      <x:c r="C17" s="50" t="str">
+        <x:v>上层应用形态</x:v>
+      </x:c>
+      <x:c r="D17" s="50" t="str">
+        <x:v>与生成式AI和CANN存在依赖关系，不能要求课程只归入一个主题</x:v>
+      </x:c>
+      <x:c r="E17" s="50" t="str">
+        <x:v>RAG应用；智能体开发；行业应用；应用评估与部署</x:v>
+      </x:c>
+      <x:c r="F17" s="50" t="str">
+        <x:v>课程主题标签；专题页；课程中心主题筛选</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="A21" s="34" t="str">
+        <x:v>3. 归类示例：一门课程使用一个主要任务和多个标签</x:v>
+      </x:c>
+      <x:c r="B21" s="34"/>
+      <x:c r="C21" s="34"/>
+      <x:c r="D21" s="34"/>
+      <x:c r="E21" s="34"/>
+    </x:row>
+    <x:row r="22" ht="32" customHeight="1">
+      <x:c r="A22" s="46" t="str">
+        <x:v>课程示例</x:v>
+      </x:c>
+      <x:c r="B22" s="47" t="str">
+        <x:v>主要开发任务</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="str">
+        <x:v>内容主题</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="str">
+        <x:v>技术栈或路线</x:v>
+      </x:c>
+      <x:c r="E22" s="48" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="58" customHeight="1">
+      <x:c r="A23" s="49" t="str">
+        <x:v>Ascend C自定义算子开发</x:v>
+      </x:c>
+      <x:c r="B23" s="49" t="str">
+        <x:v>算子开发</x:v>
+      </x:c>
+      <x:c r="C23" s="49" t="str">
+        <x:v>CANN</x:v>
+      </x:c>
+      <x:c r="D23" s="49" t="str">
+        <x:v>Ascend C</x:v>
+      </x:c>
+      <x:c r="E23" s="49" t="str">
+        <x:v>用户从算子开发入口发现，CANN用于说明内容归属</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="58" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>Triton算子开发实战</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>算子开发</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>CANN</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>Triton</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>Triton是技术路线，不与算子开发并列为一级任务</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58" customHeight="1">
+      <x:c r="A25" s="50" t="str">
+        <x:v>CPU/NPU孪生调试</x:v>
+      </x:c>
+      <x:c r="B25" s="50" t="str">
+        <x:v>调试与性能优化</x:v>
+      </x:c>
+      <x:c r="C25" s="50" t="str">
+        <x:v>CANN</x:v>
+      </x:c>
+      <x:c r="D25" s="50" t="str">
+        <x:v>Ascend C；调试工具</x:v>
+      </x:c>
+      <x:c r="E25" s="50" t="str">
+        <x:v>调试调优是主要任务，也可以出现在算子开发知识路线中</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="58" customHeight="1">
+      <x:c r="A26" s="23" t="str">
+        <x:v>大模型分布式训练</x:v>
+      </x:c>
+      <x:c r="B26" s="23" t="str">
+        <x:v>模型训练</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str">
+        <x:v>生成式AI与大模型；CANN</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="str">
+        <x:v>MindSpore；HCCL</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="str">
+        <x:v>主题允许多选，主要任务只选一个</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="58" customHeight="1">
+      <x:c r="A27" s="50" t="str">
+        <x:v>大模型推理服务部署</x:v>
+      </x:c>
+      <x:c r="B27" s="50" t="str">
+        <x:v>推理与部署</x:v>
+      </x:c>
+      <x:c r="C27" s="50" t="str">
+        <x:v>生成式AI与大模型；CANN</x:v>
+      </x:c>
+      <x:c r="D27" s="50" t="str">
+        <x:v>MindIE</x:v>
+      </x:c>
+      <x:c r="E27" s="50" t="str">
+        <x:v>避免用户在CANN和大模型主题之间二选一</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="58" customHeight="1">
+      <x:c r="A28" s="23" t="str">
+        <x:v>RAG智能体应用开发</x:v>
+      </x:c>
+      <x:c r="B28" s="23" t="str">
+        <x:v>AI应用与智能体</x:v>
+      </x:c>
+      <x:c r="C28" s="23" t="str">
+        <x:v>AI应用与智能体；生成式AI与大模型</x:v>
+      </x:c>
+      <x:c r="D28" s="23" t="str">
+        <x:v>MindIE；向量数据库；Agent框架</x:v>
+      </x:c>
+      <x:c r="E28" s="23" t="str">
+        <x:v>应用任务作为入口，模型主题和技术栈作为标签</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="28" customHeight="1">
+      <x:c r="A32" s="34" t="str">
+        <x:v>4. 分类规则与页面使用</x:v>
+      </x:c>
+      <x:c r="B32" s="34"/>
+      <x:c r="C32" s="34"/>
+    </x:row>
+    <x:row r="33" ht="32" customHeight="1">
+      <x:c r="A33" s="46" t="str">
+        <x:v>规则</x:v>
+      </x:c>
+      <x:c r="B33" s="47" t="str">
+        <x:v>具体要求</x:v>
+      </x:c>
+      <x:c r="C33" s="48" t="str">
+        <x:v>目的</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="58" customHeight="1">
+      <x:c r="A34" s="49" t="str">
+        <x:v>主要开发任务必填且单选</x:v>
+      </x:c>
+      <x:c r="B34" s="49" t="str">
+        <x:v>每门课程选择一个用户最容易理解的主要任务；跨阶段课程选择其最终要帮助用户完成的任务</x:v>
+      </x:c>
+      <x:c r="C34" s="49" t="str">
+        <x:v>保证入口和推荐结果清晰</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="58" customHeight="1">
+      <x:c r="A35" s="23" t="str">
+        <x:v>内容主题可多选</x:v>
+      </x:c>
+      <x:c r="B35" s="23" t="str">
+        <x:v>CANN、生成式AI与大模型、AI应用与智能体可同时标记</x:v>
+      </x:c>
+      <x:c r="C35" s="23" t="str">
+        <x:v>避免技术底座、模型领域和应用层互相排斥</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="58" customHeight="1">
+      <x:c r="A36" s="50" t="str">
+        <x:v>技术栈与环境可多选</x:v>
+      </x:c>
+      <x:c r="B36" s="50" t="str">
+        <x:v>记录Ascend C、Triton、CATLASS、MindSpore、MindIE、硬件和版本</x:v>
+      </x:c>
+      <x:c r="C36" s="50" t="str">
+        <x:v>支持精确筛选和兼容性判断</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="58" customHeight="1">
+      <x:c r="A37" s="23" t="str">
+        <x:v>一级任务增加一句描述</x:v>
+      </x:c>
+      <x:c r="B37" s="23" t="str">
+        <x:v>使用“用户在什么场景下，通过该分类能完成什么”描述；控制在约30字，不写技术名词堆叠</x:v>
+      </x:c>
+      <x:c r="C37" s="23" t="str">
+        <x:v>帮助不熟悉内部分类的用户快速判断</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="58" customHeight="1">
+      <x:c r="A38" s="50" t="str">
+        <x:v>二级任务按需展开</x:v>
+      </x:c>
+      <x:c r="B38" s="50" t="str">
+        <x:v>首页只展示一级任务；课程中心选择一级任务后展开二级任务；搜索自动识别同义词</x:v>
+      </x:c>
+      <x:c r="C38" s="50" t="str">
+        <x:v>兼顾易读性和精确查找</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="58" customHeight="1">
+      <x:c r="A39" s="23" t="str">
+        <x:v>新手入门不作为开发任务</x:v>
+      </x:c>
+      <x:c r="B39" s="23" t="str">
+        <x:v>作为跨任务引导入口，根据测试结果推荐训练、推理、算子或应用方向</x:v>
+      </x:c>
+      <x:c r="C39" s="23" t="str">
+        <x:v>避免把用户阶段和开发任务混为一层</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="58" customHeight="1">
+      <x:c r="A40" s="50" t="str">
+        <x:v>模型训推不作为同级分类</x:v>
+      </x:c>
+      <x:c r="B40" s="50" t="str">
+        <x:v>作为组合学习路径，内部串联训练、推理与部署内容</x:v>
+      </x:c>
+      <x:c r="C40" s="50" t="str">
+        <x:v>避免与训练开发、推理开发重复</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A4:G4"/>
+    <x:mergeCell ref="A13:F13"/>
+    <x:mergeCell ref="A21:E21"/>
+    <x:mergeCell ref="A32:C32"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: define homepage incentive leaderboard
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="Rad33e9594d444e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R199c2dd66a6d4a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="R41d5016331be4372"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="Rbfb6ef1c07ee482b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R7cc1e444a6f54431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Re72c2369e8484a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R9c18b21bb7d244af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="Rf55cf1da45ce4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R1848f2f70b914950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R94880ed586b44c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="Rbbd3f68e93454343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="R7efbd16915794c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R3cd199a4d26840a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R1304b488a7a14040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Ra79b9e8a06294889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="Rc9401c73694d4769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R6c23f1070cb442b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="Re4de62da4fdc40f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rfc451b4a6e4c49a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +61,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +91,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7F9FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF3FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E53FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -130,7 +146,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -242,6 +258,50 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -577,6 +637,471 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2E53FA"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="45" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="26" t="str">
+        <x:v>首页第三楼层｜开发者成长与贡献榜</x:v>
+      </x:c>
+      <x:c r="B1" s="27"/>
+      <x:c r="C1" s="27"/>
+      <x:c r="D1" s="27"/>
+      <x:c r="E1" s="27"/>
+      <x:c r="F1" s="27"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="28" t="str">
+        <x:v>首页展示社区榜单；个人学习反馈、下一步建议和里程碑进入个人空间或AI智能学伴。</x:v>
+      </x:c>
+      <x:c r="B2" s="27"/>
+      <x:c r="C2" s="27"/>
+      <x:c r="D2" s="27"/>
+      <x:c r="E2" s="27"/>
+      <x:c r="F2" s="27"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="55" t="str">
+        <x:v>1. 产品定位与页面边界</x:v>
+      </x:c>
+      <x:c r="B4" s="55"/>
+      <x:c r="C4" s="55"/>
+      <x:c r="D4" s="55"/>
+      <x:c r="E4" s="55"/>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="67" t="str">
+        <x:v>位置</x:v>
+      </x:c>
+      <x:c r="B5" s="68" t="str">
+        <x:v>展示内容</x:v>
+      </x:c>
+      <x:c r="C5" s="68" t="str">
+        <x:v>不展示内容</x:v>
+      </x:c>
+      <x:c r="D5" s="68" t="str">
+        <x:v>产品目的</x:v>
+      </x:c>
+      <x:c r="E5" s="69" t="str">
+        <x:v>默认范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="51" t="str">
+        <x:v>首页第三楼层</x:v>
+      </x:c>
+      <x:c r="B6" s="51" t="str">
+        <x:v>学习成长榜、实战突破榜、社区共建榜三个页签；展示排名、用户阶段、代表成果和分值或徽章</x:v>
+      </x:c>
+      <x:c r="C6" s="51" t="str">
+        <x:v>不展示‘你的本周成长’、距离下一等级、个人下一步建议等个人进度卡</x:v>
+      </x:c>
+      <x:c r="D6" s="51" t="str">
+        <x:v>让有效学习、工程实践和社区贡献被看见，为用户提供榜样与参与动机</x:v>
+      </x:c>
+      <x:c r="E6" s="51" t="str">
+        <x:v>本周榜＋同阶段用户；支持进入完整榜单</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="55" t="str">
+        <x:v>2. 首页三个榜单页签</x:v>
+      </x:c>
+      <x:c r="B9" s="55"/>
+      <x:c r="C9" s="55"/>
+      <x:c r="D9" s="55"/>
+      <x:c r="E9" s="55"/>
+      <x:c r="F9" s="55"/>
+    </x:row>
+    <x:row r="10" ht="32" customHeight="1">
+      <x:c r="A10" s="67" t="str">
+        <x:v>榜单</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="str">
+        <x:v>核心行为</x:v>
+      </x:c>
+      <x:c r="C10" s="68" t="str">
+        <x:v>核心指标</x:v>
+      </x:c>
+      <x:c r="D10" s="68" t="str">
+        <x:v>主要激励人群</x:v>
+      </x:c>
+      <x:c r="E10" s="68" t="str">
+        <x:v>首页代表成果示例</x:v>
+      </x:c>
+      <x:c r="F10" s="69" t="str">
+        <x:v>规则重点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="62" customHeight="1">
+      <x:c r="A11" s="51" t="str">
+        <x:v>学习成长榜</x:v>
+      </x:c>
+      <x:c r="B11" s="51" t="str">
+        <x:v>完成结构化学习并掌握知识</x:v>
+      </x:c>
+      <x:c r="C11" s="51" t="str">
+        <x:v>有效学习单元；首次掌握测验；按难度和规模加权的课程完成</x:v>
+      </x:c>
+      <x:c r="D11" s="51" t="str">
+        <x:v>新手；入门；学习型用户</x:v>
+      </x:c>
+      <x:c r="E11" s="51" t="str">
+        <x:v>完成分布式训练基础路径</x:v>
+      </x:c>
+      <x:c r="F11" s="51" t="str">
+        <x:v>学习时长只作个人记录；重复刷题和重复完成不重复计分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="62" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>实战突破榜</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>完成实验并解决真实开发问题</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>有效实验；经过验证的问题解决数；可复现的调试或优化结果</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>开发型用户；进阶用户</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>解决3个推理部署问题</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="str">
+        <x:v>必须包含问题、原因、解决步骤和验证结果；审核或自动验证后计分</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="62" customHeight="1">
+      <x:c r="A13" s="70" t="str">
+        <x:v>社区共建榜</x:v>
+      </x:c>
+      <x:c r="B13" s="70" t="str">
+        <x:v>纠错、抓虫并贡献可复用知识</x:v>
+      </x:c>
+      <x:c r="C13" s="70" t="str">
+        <x:v>审核通过的抓虫；有效知识贡献；被收藏、复用或官方采纳</x:v>
+      </x:c>
+      <x:c r="D13" s="70" t="str">
+        <x:v>进阶；高阶；专家</x:v>
+      </x:c>
+      <x:c r="E13" s="70" t="str">
+        <x:v>发现并推动修复高价值课程缺陷</x:v>
+      </x:c>
+      <x:c r="F13" s="70" t="str">
+        <x:v>去重、审核并按影响范围分级；数量不能代替质量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="55" t="str">
+        <x:v>3. 原始指标处理结论</x:v>
+      </x:c>
+      <x:c r="B17" s="55"/>
+      <x:c r="C17" s="55"/>
+      <x:c r="D17" s="55"/>
+      <x:c r="E17" s="55"/>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="67" t="str">
+        <x:v>原始指标</x:v>
+      </x:c>
+      <x:c r="B18" s="68" t="str">
+        <x:v>结论</x:v>
+      </x:c>
+      <x:c r="C18" s="68" t="str">
+        <x:v>最终指标或去向</x:v>
+      </x:c>
+      <x:c r="D18" s="68" t="str">
+        <x:v>原因</x:v>
+      </x:c>
+      <x:c r="E18" s="69" t="str">
+        <x:v>验证方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="62" customHeight="1">
+      <x:c r="A19" s="51" t="str">
+        <x:v>用户学习时长</x:v>
+      </x:c>
+      <x:c r="B19" s="51" t="str">
+        <x:v>降权</x:v>
+      </x:c>
+      <x:c r="C19" s="51" t="str">
+        <x:v>仅进入个人学习记录和AI智能学伴，不作为首页核心排名指标</x:v>
+      </x:c>
+      <x:c r="D19" s="51" t="str">
+        <x:v>容易挂机或被课程长度影响，不能稳定代表掌握程度</x:v>
+      </x:c>
+      <x:c r="E19" s="51" t="str">
+        <x:v>前台交互和有效学习行为可用于个人统计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="62" customHeight="1">
+      <x:c r="A20" s="23" t="str">
+        <x:v>测验通过次数</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>保留并修正</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>首次掌握知识点或首次通过测验</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>重复做简单测验会造成刷榜</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str">
+        <x:v>同一知识点首次达标计分，重复通过不重复累计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="62" customHeight="1">
+      <x:c r="A21" s="70" t="str">
+        <x:v>完成课程数</x:v>
+      </x:c>
+      <x:c r="B21" s="70" t="str">
+        <x:v>保留并加权</x:v>
+      </x:c>
+      <x:c r="C21" s="70" t="str">
+        <x:v>按课程难度、规模和完成质量计算成长值</x:v>
+      </x:c>
+      <x:c r="D21" s="70" t="str">
+        <x:v>短课程与长课程不能简单按数量等价</x:v>
+      </x:c>
+      <x:c r="E21" s="70" t="str">
+        <x:v>完成条件、关键测验和实践验收共同确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="62" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>调试错误码</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>提权并改名</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>经过验证的问题解决数</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>遇到错误不代表能力，定位并解决问题才有价值</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str">
+        <x:v>问题、根因、步骤和结果可复现或经审核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="62" customHeight="1">
+      <x:c r="A23" s="70" t="str">
+        <x:v>抓虫</x:v>
+      </x:c>
+      <x:c r="B23" s="70" t="str">
+        <x:v>重点保留</x:v>
+      </x:c>
+      <x:c r="C23" s="70" t="str">
+        <x:v>审核通过的内容纠错、课程问题、AI纠错和产品缺陷</x:v>
+      </x:c>
+      <x:c r="D23" s="70" t="str">
+        <x:v>体现社区特色，并直接改善官方学习资源质量</x:v>
+      </x:c>
+      <x:c r="E23" s="70" t="str">
+        <x:v>去重、审核、状态闭环并按影响范围分级</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="62" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>知识库建立密度</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>重新定义</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>有效知识贡献数</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>内容密度含义不清，容易鼓励堆量</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>被收录、收藏、复用、AI引用或官方标记为最佳实践</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="55" t="str">
+        <x:v>4. 计分、公平与反作弊规则</x:v>
+      </x:c>
+      <x:c r="B29" s="55"/>
+      <x:c r="C29" s="55"/>
+    </x:row>
+    <x:row r="30" ht="32" customHeight="1">
+      <x:c r="A30" s="67" t="str">
+        <x:v>规则</x:v>
+      </x:c>
+      <x:c r="B30" s="68" t="str">
+        <x:v>具体要求</x:v>
+      </x:c>
+      <x:c r="C30" s="69" t="str">
+        <x:v>解决的问题</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="54" customHeight="1">
+      <x:c r="A31" s="51" t="str">
+        <x:v>首页默认同阶段榜</x:v>
+      </x:c>
+      <x:c r="B31" s="51" t="str">
+        <x:v>新手、入门、进阶、高阶和专家优先与同阶段用户比较</x:v>
+      </x:c>
+      <x:c r="C31" s="51" t="str">
+        <x:v>避免高阶用户长期压制新手</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="54" customHeight="1">
+      <x:c r="A32" s="23" t="str">
+        <x:v>首页默认本周榜</x:v>
+      </x:c>
+      <x:c r="B32" s="23" t="str">
+        <x:v>周期结束后保留徽章或荣誉记录，排名重新开始</x:v>
+      </x:c>
+      <x:c r="C32" s="23" t="str">
+        <x:v>为新用户提供进入榜单的机会</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="54" customHeight="1">
+      <x:c r="A33" s="70" t="str">
+        <x:v>学习结果优先</x:v>
+      </x:c>
+      <x:c r="B33" s="70" t="str">
+        <x:v>按掌握、完成和验收计分，不以在线时长作为主要得分</x:v>
+      </x:c>
+      <x:c r="C33" s="70" t="str">
+        <x:v>降低挂机和无效学习</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="54" customHeight="1">
+      <x:c r="A34" s="23" t="str">
+        <x:v>同一行为不可重复得分</x:v>
+      </x:c>
+      <x:c r="B34" s="23" t="str">
+        <x:v>重复测验、重复提交、重复课程和重复缺陷不重复累计</x:v>
+      </x:c>
+      <x:c r="C34" s="23" t="str">
+        <x:v>防止刷榜</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="54" customHeight="1">
+      <x:c r="A35" s="70" t="str">
+        <x:v>贡献必须验证</x:v>
+      </x:c>
+      <x:c r="B35" s="70" t="str">
+        <x:v>抓虫和知识贡献经过自动校验、人工审核或社区采纳后计分</x:v>
+      </x:c>
+      <x:c r="C35" s="70" t="str">
+        <x:v>保证榜单可信度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="54" customHeight="1">
+      <x:c r="A36" s="23" t="str">
+        <x:v>严重程度与影响范围加权</x:v>
+      </x:c>
+      <x:c r="B36" s="23" t="str">
+        <x:v>课程无法完成、代码错误和关键版本问题高于文案纠错</x:v>
+      </x:c>
+      <x:c r="C36" s="23" t="str">
+        <x:v>奖励真正有影响力的贡献</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="55" t="str">
+        <x:v>5. 跨页面承接</x:v>
+      </x:c>
+      <x:c r="B40" s="55"/>
+      <x:c r="C40" s="55"/>
+    </x:row>
+    <x:row r="41" ht="32" customHeight="1">
+      <x:c r="A41" s="67" t="str">
+        <x:v>页面或能力</x:v>
+      </x:c>
+      <x:c r="B41" s="68" t="str">
+        <x:v>承接内容</x:v>
+      </x:c>
+      <x:c r="C41" s="69" t="str">
+        <x:v>与首页榜单的关系</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="56" customHeight="1">
+      <x:c r="A42" s="51" t="str">
+        <x:v>个人空间／我的学习</x:v>
+      </x:c>
+      <x:c r="B42" s="51" t="str">
+        <x:v>个人有效学习时长、已完成内容、成长值、徽章、历史排名</x:v>
+      </x:c>
+      <x:c r="C42" s="51" t="str">
+        <x:v>承接个人数据和长期进度，不占用首页楼层</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="56" customHeight="1">
+      <x:c r="A43" s="23" t="str">
+        <x:v>AI智能学伴</x:v>
+      </x:c>
+      <x:c r="B43" s="23" t="str">
+        <x:v>本周总结、距离下一里程碑、薄弱知识点和下一步建议</x:v>
+      </x:c>
+      <x:c r="C43" s="23" t="str">
+        <x:v>利用个人学习上下文提供动态反馈</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="56" customHeight="1">
+      <x:c r="A44" s="70" t="str">
+        <x:v>完整榜单页</x:v>
+      </x:c>
+      <x:c r="B44" s="70" t="str">
+        <x:v>时间范围、用户阶段、榜单规则、本人排名和历史荣誉</x:v>
+      </x:c>
+      <x:c r="C44" s="70" t="str">
+        <x:v>首页只展示摘要并引导查看全部</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="56" customHeight="1">
+      <x:c r="A45" s="23" t="str">
+        <x:v>课程与实验</x:v>
+      </x:c>
+      <x:c r="B45" s="23" t="str">
+        <x:v>完成条件、测验结果、实验验收和学习成果</x:v>
+      </x:c>
+      <x:c r="C45" s="23" t="str">
+        <x:v>为学习成长榜和实战突破榜提供可信数据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="56" customHeight="1">
+      <x:c r="A46" s="70" t="str">
+        <x:v>反馈与社区</x:v>
+      </x:c>
+      <x:c r="B46" s="70" t="str">
+        <x:v>抓虫提交、审核状态、知识贡献和采纳结果</x:v>
+      </x:c>
+      <x:c r="C46" s="70" t="str">
+        <x:v>为社区共建榜提供可信数据</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A4:E4"/>
+    <x:mergeCell ref="A9:F9"/>
+    <x:mergeCell ref="A17:E17"/>
+    <x:mergeCell ref="A29:C29"/>
+    <x:mergeCell ref="A40:C40"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
@@ -778,6 +1303,26 @@
       </x:c>
       <x:c r="F11" s="25" t="str">
         <x:v>进入辅助页面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="51" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="51" t="str">
+        <x:v>开发者成长与贡献榜</x:v>
+      </x:c>
+      <x:c r="C12" s="51" t="str">
+        <x:v>希望了解社区学习与贡献情况</x:v>
+      </x:c>
+      <x:c r="D12" s="51" t="str">
+        <x:v>学习成长榜、实战突破榜、社区共建榜</x:v>
+      </x:c>
+      <x:c r="E12" s="51" t="str">
+        <x:v>默认展示本周同阶段榜，可切换三个页签并进入完整榜单</x:v>
+      </x:c>
+      <x:c r="F12" s="51" t="str">
+        <x:v>发现值得学习的榜样和社区成果</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -853,13 +1398,13 @@
         <x:v>首页</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>继续学习；AI 目标输入；方向测试；AI 开发场景</x:v>
+        <x:v>继续学习；AI目标输入；方向测试；AI开发场景；开发者成长与贡献榜</x:v>
       </x:c>
       <x:c r="C5" s="24" t="str">
         <x:v>我从哪里开始？</x:v>
       </x:c>
       <x:c r="D5" s="24" t="str">
-        <x:v>示例词、标签、当前进度、六类开发场景</x:v>
+        <x:v>示例词、标签、当前进度、开发场景、本周同阶段榜单</x:v>
       </x:c>
       <x:c r="E5" s="24" t="str">
         <x:v>输入、测试、选择场景、继续学习</x:v>
@@ -1387,6 +1932,35 @@
         <x:v>所有页面使用同一份数据</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="51" t="str">
+        <x:v>M11</x:v>
+      </x:c>
+      <x:c r="B15" s="51" t="str">
+        <x:v>首页</x:v>
+      </x:c>
+      <x:c r="C15" s="51" t="str">
+        <x:v>开发者成长与贡献榜</x:v>
+      </x:c>
+      <x:c r="D15" s="51" t="str">
+        <x:v>查看同阶段开发者的学习、实战和共建成果</x:v>
+      </x:c>
+      <x:c r="E15" s="51" t="str">
+        <x:v>让有效成长和贡献被看见</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>三个榜单页签、排名、代表成果、阶段、分值或徽章</x:v>
+      </x:c>
+      <x:c r="G15" s="51" t="str">
+        <x:v>切换榜单；查看完整榜单</x:v>
+      </x:c>
+      <x:c r="H15" s="51" t="str">
+        <x:v>加载、空状态、默认页签、切换、本人未上榜</x:v>
+      </x:c>
+      <x:c r="I15" s="51" t="str">
+        <x:v>个人成长反馈进入我的学习或AI智能学伴；不在首页展示个人进度卡</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: add page design todo tracker
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R94880ed586b44c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="Rbbd3f68e93454343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="R7efbd16915794c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R3cd199a4d26840a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R1304b488a7a14040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Ra79b9e8a06294889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="Rc9401c73694d4769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R6c23f1070cb442b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="Re4de62da4fdc40f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rfc451b4a6e4c49a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R07c6995aac9d4c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R06c6465db0ec4ff0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rb0b86500921f4490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="Ree174bb7edf54f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R42d9b5a5dd0441c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Rbbd169a4dc3e49fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R5f6a0a520b2a4e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R7a47888bae154852"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R97fd00eb17554bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rc84d5656e751481a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R3ed1eb68b87f4161"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,7 +62,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -108,6 +109,16 @@
         <x:fgColor rgb="FF2E53FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E53FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -146,7 +157,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="87">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -302,6 +313,44 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -664,7 +713,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>首页展示社区榜单；个人学习反馈、下一步建议和里程碑进入个人空间或AI智能学伴。</x:v>
+        <x:v>机制方向已经确认；第三楼层的具体信息结构和交互暂挂起。个人反馈进入个人空间或AI智能学伴。</x:v>
       </x:c>
       <x:c r="B2" s="27"/>
       <x:c r="C2" s="27"/>
@@ -1098,6 +1147,650 @@
     <x:mergeCell ref="A29:C29"/>
     <x:mergeCell ref="A40:C40"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2E53FA"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="26" t="str">
+        <x:v>页面待办｜信息结构与交互</x:v>
+      </x:c>
+      <x:c r="B1" s="27"/>
+      <x:c r="C1" s="27"/>
+      <x:c r="D1" s="27"/>
+      <x:c r="E1" s="27"/>
+      <x:c r="F1" s="27"/>
+      <x:c r="G1" s="27"/>
+      <x:c r="H1" s="27"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="28" t="str">
+        <x:v>先串联主要用户流程，再逐页细化。每个页面分别维护信息结构和交互两类待办。</x:v>
+      </x:c>
+      <x:c r="B2" s="27"/>
+      <x:c r="C2" s="27"/>
+      <x:c r="D2" s="27"/>
+      <x:c r="E2" s="27"/>
+      <x:c r="F2" s="27"/>
+      <x:c r="G2" s="27"/>
+      <x:c r="H2" s="27"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="82" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="B4" s="83" t="str">
+        <x:v>页面／流程阶段</x:v>
+      </x:c>
+      <x:c r="C4" s="83" t="str">
+        <x:v>分类</x:v>
+      </x:c>
+      <x:c r="D4" s="83" t="str">
+        <x:v>当前已确认</x:v>
+      </x:c>
+      <x:c r="E4" s="83" t="str">
+        <x:v>待细化事项</x:v>
+      </x:c>
+      <x:c r="F4" s="83" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="G4" s="83" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="H4" s="84" t="str">
+        <x:v>依赖／备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="85" t="str">
+        <x:v>T001</x:v>
+      </x:c>
+      <x:c r="B5" s="85" t="str">
+        <x:v>首页</x:v>
+      </x:c>
+      <x:c r="C5" s="85" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D5" s="85" t="str">
+        <x:v>首轮保留搜索输入、开发场景、成长与贡献榜；辅助信息不设独立楼层</x:v>
+      </x:c>
+      <x:c r="E5" s="85" t="str">
+        <x:v>检查三个楼层的主次、内容密度和整体页面长度</x:v>
+      </x:c>
+      <x:c r="F5" s="85" t="str">
+        <x:v>进行中</x:v>
+      </x:c>
+      <x:c r="G5" s="85" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H5" s="85" t="str">
+        <x:v>完成主要流程后统一回看首页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>T002</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>首页</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>搜索支持输入目标、快捷方向和不知道从哪开始的测试入口</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str">
+        <x:v>搜索提交、快捷选项、场景卡及榜单入口的跳转与状态</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="str">
+        <x:v>待细化</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="str">
+        <x:v>第三楼层具体信息结构和交互暂挂起</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="86" t="str">
+        <x:v>T003</x:v>
+      </x:c>
+      <x:c r="B7" s="86" t="str">
+        <x:v>AI全屏对话／目标确认</x:v>
+      </x:c>
+      <x:c r="C7" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D7" s="86" t="str">
+        <x:v>搜索后进入全屏AI对话；追问、课程大纲和生成过程在同一条对话流中展开</x:v>
+      </x:c>
+      <x:c r="E7" s="86" t="str">
+        <x:v>定义AI首条回答、意图确认、追问问题、已确认摘要、对话阶段标识</x:v>
+      </x:c>
+      <x:c r="F7" s="86" t="str">
+        <x:v>下一步</x:v>
+      </x:c>
+      <x:c r="G7" s="86" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H7" s="86" t="str">
+        <x:v>承接首页搜索目标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="23" t="str">
+        <x:v>T004</x:v>
+      </x:c>
+      <x:c r="B8" s="23" t="str">
+        <x:v>AI全屏对话／目标确认</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="str">
+        <x:v>问题回答后自然滚动到下一问题；信息不足时动态追问</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str">
+        <x:v>定义进入方式、逐题回答、修改历史答案、跳过、返回首页、异常和中断恢复</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="str">
+        <x:v>下一步</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="str">
+        <x:v>先串主流程，再补异常流程</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="86" t="str">
+        <x:v>T005</x:v>
+      </x:c>
+      <x:c r="B9" s="86" t="str">
+        <x:v>课程大纲编辑</x:v>
+      </x:c>
+      <x:c r="C9" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D9" s="86" t="str">
+        <x:v>大纲作为AI对话中的大卡片；内部是可拖拽和滚动的画布</x:v>
+      </x:c>
+      <x:c r="E9" s="86" t="str">
+        <x:v>定义课程目标、单元、章节、依赖、内容来源、深度和环境信息</x:v>
+      </x:c>
+      <x:c r="F9" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G9" s="86" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H9" s="86" t="str">
+        <x:v>依赖目标确认结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
+      <x:c r="A10" s="23" t="str">
+        <x:v>T006</x:v>
+      </x:c>
+      <x:c r="B10" s="23" t="str">
+        <x:v>课程大纲编辑</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="str">
+        <x:v>支持全屏查看、编辑节点、增加章节、调整学习深浅</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str">
+        <x:v>定义画布拖拽缩放、节点选中、增删改、撤销、保存和确认</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="str">
+        <x:v>确认后进入课程生成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
+      <x:c r="A11" s="86" t="str">
+        <x:v>T007</x:v>
+      </x:c>
+      <x:c r="B11" s="86" t="str">
+        <x:v>课程生成过程</x:v>
+      </x:c>
+      <x:c r="C11" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D11" s="86" t="str">
+        <x:v>大纲确认后继续在AI对话中生成课程；课程预览逐步出现</x:v>
+      </x:c>
+      <x:c r="E11" s="86" t="str">
+        <x:v>定义生成进度、正在生成的单元、来源校验、失败提示和可预览范围</x:v>
+      </x:c>
+      <x:c r="F11" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G11" s="86" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H11" s="86" t="str">
+        <x:v>课程内容采用打字机式出现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
+      <x:c r="A12" s="23" t="str">
+        <x:v>T008</x:v>
+      </x:c>
+      <x:c r="B12" s="23" t="str">
+        <x:v>课程生成过程</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="str">
+        <x:v>课程内容一边生成一边写入纸张式预览</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str">
+        <x:v>定义暂停、继续、取消、后台生成、离开恢复和局部失败重试</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="str">
+        <x:v>生成完成后进入独立预览</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
+      <x:c r="A13" s="86" t="str">
+        <x:v>T009</x:v>
+      </x:c>
+      <x:c r="B13" s="86" t="str">
+        <x:v>课程预览</x:v>
+      </x:c>
+      <x:c r="C13" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D13" s="86" t="str">
+        <x:v>进入沉浸学习前提供独立课程概览</x:v>
+      </x:c>
+      <x:c r="E13" s="86" t="str">
+        <x:v>定义适合人群、成果、知识路线、学习成本、环境、来源、版本和目录摘要</x:v>
+      </x:c>
+      <x:c r="F13" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G13" s="86" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H13" s="86" t="str">
+        <x:v>与首页课程卡信息保持一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
+      <x:c r="A14" s="23" t="str">
+        <x:v>T010</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>课程预览</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="str">
+        <x:v>用户了解课程后再进入学习</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="str">
+        <x:v>定义开始学习、返回修改大纲、收藏、分享和来源异常处理</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="str">
+        <x:v>进入沉浸式学习</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
+      <x:c r="A15" s="86" t="str">
+        <x:v>T011</x:v>
+      </x:c>
+      <x:c r="B15" s="86" t="str">
+        <x:v>沉浸式学习</x:v>
+      </x:c>
+      <x:c r="C15" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D15" s="86" t="str">
+        <x:v>支持视频、白板、图文、代码、资料、测验和AI助手</x:v>
+      </x:c>
+      <x:c r="E15" s="86" t="str">
+        <x:v>定义章节导航、主学习区、代码区、资料区、验收和上下文信息</x:v>
+      </x:c>
+      <x:c r="F15" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G15" s="86" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H15" s="86" t="str">
+        <x:v>需区分视频与白板两种主视图</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>T012</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>沉浸式学习</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>支持视图切换、代码运行、笔记和AI问答</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str">
+        <x:v>定义播放与代码联动、白板操作、运行反馈、进度保存和跨设备恢复</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="str">
+        <x:v>依赖学习单元结构</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="86" t="str">
+        <x:v>T013</x:v>
+      </x:c>
+      <x:c r="B17" s="86" t="str">
+        <x:v>我的学习／个人空间</x:v>
+      </x:c>
+      <x:c r="C17" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D17" s="86" t="str">
+        <x:v>承接计划、进度、能力、笔记、实践、认证及个人激励反馈</x:v>
+      </x:c>
+      <x:c r="E17" s="86" t="str">
+        <x:v>定义进行中、已完成、待复习、能力图谱、徽章和历史排名</x:v>
+      </x:c>
+      <x:c r="F17" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G17" s="86" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H17" s="86" t="str">
+        <x:v>不在首页展示个人成长卡</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="23" t="str">
+        <x:v>T014</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>我的学习／个人空间</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="str">
+        <x:v>支持继续学习和回看个人成长</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="str">
+        <x:v>定义筛选、继续学习、复习、查看成果和管理计划</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="str">
+        <x:v>与AI智能学伴共享数据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="86" t="str">
+        <x:v>T015</x:v>
+      </x:c>
+      <x:c r="B19" s="86" t="str">
+        <x:v>AI智能学伴</x:v>
+      </x:c>
+      <x:c r="C19" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D19" s="86" t="str">
+        <x:v>使用学习上下文提供总结、解释、排错和下一步建议</x:v>
+      </x:c>
+      <x:c r="E19" s="86" t="str">
+        <x:v>定义上下文范围、引用来源、个人总结、里程碑和推荐内容</x:v>
+      </x:c>
+      <x:c r="F19" s="86" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G19" s="86" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H19" s="86" t="str">
+        <x:v>跨页能力</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="64" customHeight="1">
+      <x:c r="A20" s="23" t="str">
+        <x:v>T016</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>AI智能学伴</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="str">
+        <x:v>可从学习过程或个人空间唤起</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str">
+        <x:v>定义入口、展开方式、上下文切换、引用跳转和反馈</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="str">
+        <x:v>避免遮挡当前学习任务</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="64" customHeight="1">
+      <x:c r="A21" s="86" t="str">
+        <x:v>T017</x:v>
+      </x:c>
+      <x:c r="B21" s="86" t="str">
+        <x:v>开发场景／全部资源</x:v>
+      </x:c>
+      <x:c r="C21" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D21" s="86" t="str">
+        <x:v>按主要开发任务和内容主题组织可信资源</x:v>
+      </x:c>
+      <x:c r="E21" s="86" t="str">
+        <x:v>定义筛选器、任务路线、课程卡、资源来源和环境标签</x:v>
+      </x:c>
+      <x:c r="F21" s="86" t="str">
+        <x:v>部分确认</x:v>
+      </x:c>
+      <x:c r="G21" s="86" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H21" s="86" t="str">
+        <x:v>主要任务与内容主题分类已确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="64" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>T018</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>开发场景／全部资源</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>支持筛选、比较并进入课程预览或AI生成</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str">
+        <x:v>定义筛选联动、排序、卡片悬浮、查看全部和无结果推荐</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="str">
+        <x:v>待细化</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="str">
+        <x:v>课程卡默认与悬浮结构待最终确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="64" customHeight="1">
+      <x:c r="A23" s="86" t="str">
+        <x:v>T019</x:v>
+      </x:c>
+      <x:c r="B23" s="86" t="str">
+        <x:v>开发者成长与贡献榜</x:v>
+      </x:c>
+      <x:c r="C23" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D23" s="86" t="str">
+        <x:v>三个榜单及其指标、验证和反作弊原则已确认</x:v>
+      </x:c>
+      <x:c r="E23" s="86" t="str">
+        <x:v>定义首页榜单行、完整榜单字段和规则说明</x:v>
+      </x:c>
+      <x:c r="F23" s="86" t="str">
+        <x:v>暂挂</x:v>
+      </x:c>
+      <x:c r="G23" s="86" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H23" s="86" t="str">
+        <x:v>完成主要学习流程后恢复</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="64" customHeight="1">
+      <x:c r="A24" s="23" t="str">
+        <x:v>T020</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>开发者成长与贡献榜</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="str">
+        <x:v>首页仅呈现榜单摘要，不呈现个人进度卡</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str">
+        <x:v>定义页签切换、时间和阶段筛选、查看全部及异常状态</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="str">
+        <x:v>暂挂</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="str">
+        <x:v>完成主要学习流程后恢复</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="64" customHeight="1">
+      <x:c r="A25" s="86" t="str">
+        <x:v>T021</x:v>
+      </x:c>
+      <x:c r="B25" s="86" t="str">
+        <x:v>社区与帮助</x:v>
+      </x:c>
+      <x:c r="C25" s="86" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D25" s="86" t="str">
+        <x:v>承接案例、讨论、反馈和抓虫</x:v>
+      </x:c>
+      <x:c r="E25" s="86" t="str">
+        <x:v>定义抓虫提交、审核状态、问题案例和帮助内容</x:v>
+      </x:c>
+      <x:c r="F25" s="86" t="str">
+        <x:v>后续</x:v>
+      </x:c>
+      <x:c r="G25" s="86" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H25" s="86" t="str">
+        <x:v>与社区共建榜关联</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="64" customHeight="1">
+      <x:c r="A26" s="23" t="str">
+        <x:v>T022</x:v>
+      </x:c>
+      <x:c r="B26" s="23" t="str">
+        <x:v>社区与帮助</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="str">
+        <x:v>支持提交反馈并追踪处理结果</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="str">
+        <x:v>定义提交、补充证据、去重提示、审核和状态通知</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="str">
+        <x:v>后续</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H26" s="23" t="str">
+        <x:v>首轮仅保留必要反馈入口</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1290,7 +1983,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="25" t="str">
-        <x:v>辅助入口</x:v>
+        <x:v>辅助入口（首轮不设独立楼层）</x:v>
       </x:c>
       <x:c r="C11" s="25" t="str">
         <x:v>明确需要资源或帮助</x:v>
@@ -1299,7 +1992,7 @@
         <x:v>全部官方资源、认证、社区与帮助</x:v>
       </x:c>
       <x:c r="E11" s="25" t="str">
-        <x:v>放在导航或页面较低位置</x:v>
+        <x:v>首轮仅由顶部导航或页脚承接，不占用首页楼层</x:v>
       </x:c>
       <x:c r="F11" s="25" t="str">
         <x:v>进入辅助页面</x:v>
@@ -1955,10 +2648,10 @@
         <x:v>切换榜单；查看完整榜单</x:v>
       </x:c>
       <x:c r="H15" s="51" t="str">
-        <x:v>加载、空状态、默认页签、切换、本人未上榜</x:v>
+        <x:v>具体信息结构和交互暂挂起</x:v>
       </x:c>
       <x:c r="I15" s="51" t="str">
-        <x:v>个人成长反馈进入我的学习或AI智能学伴；不在首页展示个人进度卡</x:v>
+        <x:v>保留产品机制定义；个人反馈进入我的学习或AI智能学伴</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: add leaderboard placeholder copy
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R07c6995aac9d4c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R06c6465db0ec4ff0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rb0b86500921f4490"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="Ree174bb7edf54f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R42d9b5a5dd0441c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Rbbd169a4dc3e49fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R5f6a0a520b2a4e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R7a47888bae154852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R97fd00eb17554bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rc84d5656e751481a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R3ed1eb68b87f4161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R3029e95a727d4b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R6103525cd0104f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rd150b19bd96042e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R7af25642d9054763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="Rf3e4a656ffd84637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Re2c9cb22a1994b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R3b41522756384c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R04387d29d5b740f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R5bacce9348a447a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="R2b73a67655314b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R1501795f93ed4628"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -62,7 +62,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +119,21 @@
         <x:fgColor rgb="FFF7F9FF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF3FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E53FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -157,7 +172,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -351,6 +366,50 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1139,6 +1198,185 @@
         <x:v>为社区共建榜提供可信数据</x:v>
       </x:c>
     </x:row>
+    <x:row r="49" ht="28" customHeight="1">
+      <x:c r="A49" s="90" t="str">
+        <x:v>6. 首页榜单占位文案</x:v>
+      </x:c>
+      <x:c r="B49" s="90"/>
+      <x:c r="C49" s="90"/>
+      <x:c r="D49" s="90"/>
+      <x:c r="E49" s="90"/>
+    </x:row>
+    <x:row r="50" ht="32" customHeight="1">
+      <x:c r="A50" s="102" t="str">
+        <x:v>榜单</x:v>
+      </x:c>
+      <x:c r="B50" s="103" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="C50" s="103" t="str">
+        <x:v>用户名</x:v>
+      </x:c>
+      <x:c r="D50" s="103" t="str">
+        <x:v>用户行为</x:v>
+      </x:c>
+      <x:c r="E50" s="104" t="str">
+        <x:v>文案规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="48" customHeight="1">
+      <x:c r="A51" s="105" t="str">
+        <x:v>学习成长榜</x:v>
+      </x:c>
+      <x:c r="B51" s="105" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="C51" s="105" t="str">
+        <x:v>MindSpore小林</x:v>
+      </x:c>
+      <x:c r="D51" s="105" t="str">
+        <x:v>完成「分布式训练基础」学习路径并通过结课测验</x:v>
+      </x:c>
+      <x:c r="E51" s="105" t="str">
+        <x:v>突出完成对象和掌握结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="48" customHeight="1">
+      <x:c r="A52" s="23" t="str">
+        <x:v>学习成长榜</x:v>
+      </x:c>
+      <x:c r="B52" s="23" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="C52" s="23" t="str">
+        <x:v>昇腾新手阿杰</x:v>
+      </x:c>
+      <x:c r="D52" s="23" t="str">
+        <x:v>本周完成6个学习单元，首次掌握12个知识点</x:v>
+      </x:c>
+      <x:c r="E52" s="23" t="str">
+        <x:v>避免只展示在线时长</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="48" customHeight="1">
+      <x:c r="A53" s="106" t="str">
+        <x:v>学习成长榜</x:v>
+      </x:c>
+      <x:c r="B53" s="106" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="C53" s="106" t="str">
+        <x:v>模型训练笔记</x:v>
+      </x:c>
+      <x:c r="D53" s="106" t="str">
+        <x:v>完成大模型训练入门课程及3次配套实验</x:v>
+      </x:c>
+      <x:c r="E53" s="106" t="str">
+        <x:v>课程和实践可以同时出现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="48" customHeight="1">
+      <x:c r="A54" s="23" t="str">
+        <x:v>实战突破榜</x:v>
+      </x:c>
+      <x:c r="B54" s="23" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="C54" s="23" t="str">
+        <x:v>NPU调优手记</x:v>
+      </x:c>
+      <x:c r="D54" s="23" t="str">
+        <x:v>定位并解决3个推理部署问题，方案均已验证</x:v>
+      </x:c>
+      <x:c r="E54" s="23" t="str">
+        <x:v>强调问题已经解决和验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="48" customHeight="1">
+      <x:c r="A55" s="106" t="str">
+        <x:v>实战突破榜</x:v>
+      </x:c>
+      <x:c r="B55" s="106" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="C55" s="106" t="str">
+        <x:v>算子工坊Leo</x:v>
+      </x:c>
+      <x:c r="D55" s="106" t="str">
+        <x:v>完成Ascend C自定义算子的开发、运行与精度验证</x:v>
+      </x:c>
+      <x:c r="E55" s="106" t="str">
+        <x:v>展示完整工程结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="48" customHeight="1">
+      <x:c r="A56" s="23" t="str">
+        <x:v>实战突破榜</x:v>
+      </x:c>
+      <x:c r="B56" s="23" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="C56" s="23" t="str">
+        <x:v>HCCL观察员</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="str">
+        <x:v>解决多卡训练通信超时，使训练任务恢复运行</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="str">
+        <x:v>突出问题场景和最终结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="48" customHeight="1">
+      <x:c r="A57" s="106" t="str">
+        <x:v>社区共建榜</x:v>
+      </x:c>
+      <x:c r="B57" s="106" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="C57" s="106" t="str">
+        <x:v>CANN捕虫者</x:v>
+      </x:c>
+      <x:c r="D57" s="106" t="str">
+        <x:v>发现课程代码的版本兼容问题并推动完成修复</x:v>
+      </x:c>
+      <x:c r="E57" s="106" t="str">
+        <x:v>抓虫必须体现处理结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="48" customHeight="1">
+      <x:c r="A58" s="23" t="str">
+        <x:v>社区共建榜</x:v>
+      </x:c>
+      <x:c r="B58" s="23" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="C58" s="23" t="str">
+        <x:v>文档修补匠</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="str">
+        <x:v>贡献OOM排查最佳实践，已被官方知识库收录</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="str">
+        <x:v>强调贡献被采用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="48" customHeight="1">
+      <x:c r="A59" s="106" t="str">
+        <x:v>社区共建榜</x:v>
+      </x:c>
+      <x:c r="B59" s="106" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="C59" s="106" t="str">
+        <x:v>AI纠错员</x:v>
+      </x:c>
+      <x:c r="D59" s="106" t="str">
+        <x:v>纠正AI回答中的接口版本错误，帮助更新引用来源</x:v>
+      </x:c>
+      <x:c r="E59" s="106" t="str">
+        <x:v>说明纠错对象和社区价值</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A4:E4"/>
@@ -1146,6 +1384,7 @@
     <x:mergeCell ref="A17:E17"/>
     <x:mergeCell ref="A29:C29"/>
     <x:mergeCell ref="A40:C40"/>
+    <x:mergeCell ref="A49:E49"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1697,7 +1936,7 @@
         <x:v>信息结构</x:v>
       </x:c>
       <x:c r="D23" s="86" t="str">
-        <x:v>三个榜单及其指标、验证和反作弊原则已确认</x:v>
+        <x:v>三个榜单及指标、验证和反作弊原则已确认；首页占位用户名和行为文案已补充</x:v>
       </x:c>
       <x:c r="E23" s="86" t="str">
         <x:v>定义首页榜单行、完整榜单字段和规则说明</x:v>

</xml_diff>

<commit_message>
docs: record video learning workspace decisions
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R3029e95a727d4b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R6103525cd0104f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rd150b19bd96042e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R7af25642d9054763"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="Rf3e4a656ffd84637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="Re2c9cb22a1994b70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R3b41522756384c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="R04387d29d5b740f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R5bacce9348a447a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="R2b73a67655314b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R1501795f93ed4628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R107f5bd5647747d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="Rbd032eed093a4a6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rcb775c0ad07e49bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R4b453b14a1924e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="Rd99ec06a50b64f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="R3a37ca6945eb4c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R0c8458ab0e654431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="Rebb174f090d14b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R5baae03f58ee4ad9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rc5510a9224c24e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R1377e6d99eca47d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1728,19 +1728,19 @@
         <x:v>信息结构</x:v>
       </x:c>
       <x:c r="D15" s="86" t="str">
-        <x:v>支持视频、白板、图文、代码、资料、测验和AI助手</x:v>
+        <x:v>视频学习采用浅色可调工作台；顶部沿用关闭、课节标题、视频／白板切换和辅助工具；主体为视频、视频代码、IDE三张卡片</x:v>
       </x:c>
       <x:c r="E15" s="86" t="str">
-        <x:v>定义章节导航、主学习区、代码区、资料区、验收和上下文信息</x:v>
+        <x:v>补充真实视频源、字幕、章节导航、错误码、测验和相关文档的数据结构</x:v>
       </x:c>
       <x:c r="F15" s="86" t="str">
-        <x:v>待开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="G15" s="86" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H15" s="86" t="str">
-        <x:v>需区分视频与白板两种主视图</x:v>
+        <x:v>视频区域默认最大；三张卡片圆角12px、间距8px；IDE位于右侧</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -1754,19 +1754,19 @@
         <x:v>交互</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>支持视图切换、代码运行、笔记和AI问答</x:v>
+        <x:v>视频与白板可切换；代码时间点联动视频；代码支持复制、AI解读和置入IDE；三栏可拖动调宽，IDE可收起</x:v>
       </x:c>
       <x:c r="E16" s="23" t="str">
-        <x:v>定义播放与代码联动、白板操作、运行反馈、进度保存和跨设备恢复</x:v>
+        <x:v>补充真实播放控制、拖动布局持久化、IDE运行反馈、学习进度保存和异常恢复</x:v>
       </x:c>
       <x:c r="F16" s="23" t="str">
-        <x:v>待开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="G16" s="23" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H16" s="23" t="str">
-        <x:v>依赖学习单元结构</x:v>
+        <x:v>拖动分隔条支持左右方向键；移动端自动改为单列排列</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">

</xml_diff>

<commit_message>
docs: map feedback incentive touchpoints
</commit_message>
<xml_diff>
--- a/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
+++ b/outputs/product-structure-prd/开发者学习平台产品结构.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R107f5bd5647747d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="Rbd032eed093a4a6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rcb775c0ad07e49bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R4b453b14a1924e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="Rd99ec06a50b64f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="R3a37ca6945eb4c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="R0c8458ab0e654431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="Rebb174f090d14b10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R5baae03f58ee4ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rc5510a9224c24e0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="R1377e6d99eca47d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品总览" sheetId="1" r:id="R86adbb83a1354001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首页入口" sheetId="2" r:id="R84551cd4f3314983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面地图" sheetId="3" r:id="Rbeda2b15ac444c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块设计" sheetId="4" r:id="R91639041231d49b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学习单元" sheetId="5" r:id="R3a183f6ecbf34f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容来源" sheetId="6" r:id="R24e54acf1c06429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨页能力" sheetId="7" r:id="Rbfa257487544472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实施计划" sheetId="8" r:id="Reffe7c5adf3e497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类体系" sheetId="9" r:id="R6273d8de7b56407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激励机制" sheetId="10" r:id="Rbe33263fb74b4cf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面待办" sheetId="11" r:id="Rf9accd2eff414303"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="反馈激励触点地图" sheetId="12" r:id="R796338dde50b46f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,8 +62,19 @@
       <x:color rgb="FF101828"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF172554"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF667085"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -134,6 +146,16 @@
         <x:fgColor rgb="FFF7F9FF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E53FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -172,7 +194,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="107">
+  <x:cellXfs count="117">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -410,6 +432,28 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -772,7 +816,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>机制方向已经确认；第三楼层的具体信息结构和交互暂挂起。个人反馈进入个人空间或AI智能学伴。</x:v>
+        <x:v>机制方向更新：开发者成长属于面向开发者的反馈与激励体系。首页保留公共榜单摘要；需继续研究学习生成、沉浸学习、IDE实践、社区贡献、个人空间与AI学伴等触点。</x:v>
       </x:c>
       <x:c r="B2" s="27"/>
       <x:c r="C2" s="27"/>
@@ -858,16 +902,16 @@
         <x:v>学习成长榜</x:v>
       </x:c>
       <x:c r="B11" s="51" t="str">
-        <x:v>完成结构化学习并掌握知识</x:v>
+        <x:v>结构化学习→能力掌握→实验验证</x:v>
       </x:c>
       <x:c r="C11" s="51" t="str">
-        <x:v>有效学习单元；首次掌握测验；按难度和规模加权的课程完成</x:v>
+        <x:v>完成学习路径；首次掌握知识点；关键实验通过；按难度和规模加权的有效成长值</x:v>
       </x:c>
       <x:c r="D11" s="51" t="str">
-        <x:v>新手；入门；学习型用户</x:v>
+        <x:v>新手、入门和希望建立开发基础的用户</x:v>
       </x:c>
       <x:c r="E11" s="51" t="str">
-        <x:v>完成分布式训练基础路径</x:v>
+        <x:v>展示学习阶段、已掌握能力和代表性实践，不以在线时长或课程数量单独排名</x:v>
       </x:c>
       <x:c r="F11" s="51" t="str">
         <x:v>学习时长只作个人记录；重复刷题和重复完成不重复计分</x:v>
@@ -878,16 +922,16 @@
         <x:v>实战突破榜</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
-        <x:v>完成实验并解决真实开发问题</x:v>
+        <x:v>把课程知识用于真实开发任务并完成验收</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
-        <x:v>有效实验；经过验证的问题解决数；可复现的调试或优化结果</x:v>
+        <x:v>有效问题解决；调试结果可复现；性能、精度或稳定性改善；真实任务验收</x:v>
       </x:c>
       <x:c r="D12" s="23" t="str">
-        <x:v>开发型用户；进阶用户</x:v>
+        <x:v>进阶开发者和正在处理项目问题的用户</x:v>
       </x:c>
       <x:c r="E12" s="23" t="str">
-        <x:v>解决3个推理部署问题</x:v>
+        <x:v>展示问题场景、解决结果和验证证据，不以遇到错误数排名</x:v>
       </x:c>
       <x:c r="F12" s="23" t="str">
         <x:v>必须包含问题、原因、解决步骤和验证结果；审核或自动验证后计分</x:v>
@@ -898,16 +942,16 @@
         <x:v>社区共建榜</x:v>
       </x:c>
       <x:c r="B13" s="70" t="str">
-        <x:v>纠错、抓虫并贡献可复用知识</x:v>
+        <x:v>把纠错、抓虫和经验沉淀为可复用知识</x:v>
       </x:c>
       <x:c r="C13" s="70" t="str">
-        <x:v>审核通过的抓虫；有效知识贡献；被收藏、复用或官方采纳</x:v>
+        <x:v>审核通过；官方采纳；被收藏、引用或复用；影响范围；问题闭环</x:v>
       </x:c>
       <x:c r="D13" s="70" t="str">
-        <x:v>进阶；高阶；专家</x:v>
+        <x:v>愿意改善内容和帮助他人的用户</x:v>
       </x:c>
       <x:c r="E13" s="70" t="str">
-        <x:v>发现并推动修复高价值课程缺陷</x:v>
+        <x:v>展示贡献类型、处理结果和被采用证据，不以提交数量单独排名</x:v>
       </x:c>
       <x:c r="F13" s="70" t="str">
         <x:v>去重、审核并按影响范围分级；数量不能代替质量</x:v>
@@ -1200,7 +1244,7 @@
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="90" t="str">
-        <x:v>6. 首页榜单占位文案</x:v>
+        <x:v>6. 首页榜单展示规则</x:v>
       </x:c>
       <x:c r="B49" s="90"/>
       <x:c r="C49" s="90"/>
@@ -1212,16 +1256,16 @@
         <x:v>榜单</x:v>
       </x:c>
       <x:c r="B50" s="103" t="str">
-        <x:v>排名</x:v>
+        <x:v>学习场景关联</x:v>
       </x:c>
       <x:c r="C50" s="103" t="str">
-        <x:v>用户名</x:v>
+        <x:v>首页卡片显示</x:v>
       </x:c>
       <x:c r="D50" s="103" t="str">
-        <x:v>用户行为</x:v>
+        <x:v>排名依据</x:v>
       </x:c>
       <x:c r="E50" s="104" t="str">
-        <x:v>文案规则</x:v>
+        <x:v>点击后</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
@@ -1229,153 +1273,113 @@
         <x:v>学习成长榜</x:v>
       </x:c>
       <x:c r="B51" s="105" t="str">
-        <x:v>01</x:v>
+        <x:v>完成路径并掌握知识</x:v>
       </x:c>
       <x:c r="C51" s="105" t="str">
-        <x:v>MindSpore小林</x:v>
+        <x:v>用户名、当前阶段、代表性学习成果、有效成长值</x:v>
       </x:c>
       <x:c r="D51" s="105" t="str">
-        <x:v>完成「分布式训练基础」学习路径并通过结课测验</x:v>
+        <x:v>掌握与验证优先；同阶段、本周周期</x:v>
       </x:c>
       <x:c r="E51" s="105" t="str">
-        <x:v>突出完成对象和掌握结果</x:v>
+        <x:v>进入完整榜单或个人成长证据</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" s="23" t="str">
-        <x:v>学习成长榜</x:v>
+        <x:v>实战突破榜</x:v>
       </x:c>
       <x:c r="B52" s="23" t="str">
-        <x:v>02</x:v>
+        <x:v>完成实验并解决真实开发问题</x:v>
       </x:c>
       <x:c r="C52" s="23" t="str">
-        <x:v>昇腾新手阿杰</x:v>
+        <x:v>用户名、问题场景、解决结果、验证标签</x:v>
       </x:c>
       <x:c r="D52" s="23" t="str">
-        <x:v>本周完成6个学习单元，首次掌握12个知识点</x:v>
+        <x:v>问题解决质量、结果影响和可复现性</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
-        <x:v>避免只展示在线时长</x:v>
+        <x:v>进入问题案例或实践详情</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" s="106" t="str">
-        <x:v>学习成长榜</x:v>
+        <x:v>社区共建榜</x:v>
       </x:c>
       <x:c r="B53" s="106" t="str">
-        <x:v>03</x:v>
+        <x:v>纠错、抓虫并贡献可复用知识</x:v>
       </x:c>
       <x:c r="C53" s="106" t="str">
-        <x:v>模型训练笔记</x:v>
+        <x:v>用户名、贡献类型、处理状态、采用／复用证据</x:v>
       </x:c>
       <x:c r="D53" s="106" t="str">
-        <x:v>完成大模型训练入门课程及3次配套实验</x:v>
+        <x:v>审核、采纳、复用和影响范围</x:v>
       </x:c>
       <x:c r="E53" s="106" t="str">
-        <x:v>课程和实践可以同时出现</x:v>
+        <x:v>进入贡献详情、社区案例或反馈记录</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" s="23" t="str">
-        <x:v>实战突破榜</x:v>
+        <x:v>统一呈现</x:v>
       </x:c>
       <x:c r="B54" s="23" t="str">
-        <x:v>01</x:v>
+        <x:v>三个榜单均回到真实学习或开发任务</x:v>
       </x:c>
       <x:c r="C54" s="23" t="str">
-        <x:v>NPU调优手记</x:v>
+        <x:v>默认本周、同阶段、三条代表记录；不展示个人成长卡</x:v>
       </x:c>
       <x:c r="D54" s="23" t="str">
-        <x:v>定位并解决3个推理部署问题，方案均已验证</x:v>
+        <x:v>不使用单一总分；每榜单使用自己的证据规则</x:v>
       </x:c>
       <x:c r="E54" s="23" t="str">
-        <x:v>强调问题已经解决和验证</x:v>
+        <x:v>查看完整榜单、规则和个人空间</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" s="106" t="str">
-        <x:v>实战突破榜</x:v>
+        <x:v>首页边界</x:v>
       </x:c>
       <x:c r="B55" s="106" t="str">
-        <x:v>02</x:v>
+        <x:v>首页是公共反馈触点</x:v>
       </x:c>
       <x:c r="C55" s="106" t="str">
-        <x:v>算子工坊Leo</x:v>
+        <x:v>只展示榜单摘要和榜样行为</x:v>
       </x:c>
       <x:c r="D55" s="106" t="str">
-        <x:v>完成Ascend C自定义算子的开发、运行与精度验证</x:v>
+        <x:v>个人进度、薄弱点和下一步行动不在首页展开</x:v>
       </x:c>
       <x:c r="E55" s="106" t="str">
-        <x:v>展示完整工程结果</x:v>
+        <x:v>转入我的学习、AI学伴或具体任务页</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
-      <x:c r="A56" s="23" t="str">
-        <x:v>实战突破榜</x:v>
-      </x:c>
-      <x:c r="B56" s="23" t="str">
-        <x:v>03</x:v>
-      </x:c>
-      <x:c r="C56" s="23" t="str">
-        <x:v>HCCL观察员</x:v>
-      </x:c>
-      <x:c r="D56" s="23" t="str">
-        <x:v>解决多卡训练通信超时，使训练任务恢复运行</x:v>
-      </x:c>
-      <x:c r="E56" s="23" t="str">
-        <x:v>突出问题场景和最终结果</x:v>
-      </x:c>
+      <x:c r="A56" s="23"/>
+      <x:c r="B56" s="23"/>
+      <x:c r="C56" s="23"/>
+      <x:c r="D56" s="23"/>
+      <x:c r="E56" s="23"/>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
-      <x:c r="A57" s="106" t="str">
-        <x:v>社区共建榜</x:v>
-      </x:c>
-      <x:c r="B57" s="106" t="str">
-        <x:v>01</x:v>
-      </x:c>
-      <x:c r="C57" s="106" t="str">
-        <x:v>CANN捕虫者</x:v>
-      </x:c>
-      <x:c r="D57" s="106" t="str">
-        <x:v>发现课程代码的版本兼容问题并推动完成修复</x:v>
-      </x:c>
-      <x:c r="E57" s="106" t="str">
-        <x:v>抓虫必须体现处理结果</x:v>
-      </x:c>
+      <x:c r="A57" s="106"/>
+      <x:c r="B57" s="106"/>
+      <x:c r="C57" s="106"/>
+      <x:c r="D57" s="106"/>
+      <x:c r="E57" s="106"/>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
-      <x:c r="A58" s="23" t="str">
-        <x:v>社区共建榜</x:v>
-      </x:c>
-      <x:c r="B58" s="23" t="str">
-        <x:v>02</x:v>
-      </x:c>
-      <x:c r="C58" s="23" t="str">
-        <x:v>文档修补匠</x:v>
-      </x:c>
-      <x:c r="D58" s="23" t="str">
-        <x:v>贡献OOM排查最佳实践，已被官方知识库收录</x:v>
-      </x:c>
-      <x:c r="E58" s="23" t="str">
-        <x:v>强调贡献被采用</x:v>
-      </x:c>
+      <x:c r="A58" s="23"/>
+      <x:c r="B58" s="23"/>
+      <x:c r="C58" s="23"/>
+      <x:c r="D58" s="23"/>
+      <x:c r="E58" s="23"/>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
-      <x:c r="A59" s="106" t="str">
-        <x:v>社区共建榜</x:v>
-      </x:c>
-      <x:c r="B59" s="106" t="str">
-        <x:v>03</x:v>
-      </x:c>
-      <x:c r="C59" s="106" t="str">
-        <x:v>AI纠错员</x:v>
-      </x:c>
-      <x:c r="D59" s="106" t="str">
-        <x:v>纠正AI回答中的接口版本错误，帮助更新引用来源</x:v>
-      </x:c>
-      <x:c r="E59" s="106" t="str">
-        <x:v>说明纠错对象和社区价值</x:v>
-      </x:c>
+      <x:c r="A59" s="106"/>
+      <x:c r="B59" s="106"/>
+      <x:c r="C59" s="106"/>
+      <x:c r="D59" s="106"/>
+      <x:c r="E59" s="106"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1936,19 +1940,19 @@
         <x:v>信息结构</x:v>
       </x:c>
       <x:c r="D23" s="86" t="str">
-        <x:v>三个榜单及指标、验证和反作弊原则已确认；首页占位用户名和行为文案已补充</x:v>
+        <x:v>开发者成长重新定义为反馈与激励体系；首页保留学习成长、实战突破和社区共建的公共榜单摘要</x:v>
       </x:c>
       <x:c r="E23" s="86" t="str">
-        <x:v>定义首页榜单行、完整榜单字段和规则说明</x:v>
+        <x:v>开展竞品分析，判断首页榜单应展示的反馈、证明和下一步行动</x:v>
       </x:c>
       <x:c r="F23" s="86" t="str">
-        <x:v>暂挂</x:v>
+        <x:v>调研中</x:v>
       </x:c>
       <x:c r="G23" s="86" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="H23" s="86" t="str">
-        <x:v>完成主要学习流程后恢复</x:v>
+        <x:v>首页负责公共反馈与榜样发现；个人反馈不集中堆在首页</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
@@ -1962,19 +1966,19 @@
         <x:v>交互</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>首页仅呈现榜单摘要，不呈现个人进度卡</x:v>
+        <x:v>首页只承担反馈与激励体系的一个触点，完整机制需要覆盖主要用户流程</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>定义页签切换、时间和阶段筛选、查看全部及异常状态</x:v>
+        <x:v>定义首页摘要与完整榜单的进入方式，并与学习、实践、社区和个人空间衔接</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
-        <x:v>暂挂</x:v>
+        <x:v>调研中</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="H24" s="23" t="str">
-        <x:v>完成主要学习流程后恢复</x:v>
+        <x:v>先完成跨页面触点地图，再细化首页交互</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="64" customHeight="1">
@@ -2029,7 +2033,290 @@
         <x:v>首轮仅保留必要反馈入口</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>T023</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>全站反馈与激励触点</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>信息结构</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>反馈与激励不能只放在首页，需要覆盖学习、实践和社区共建的关键阶段</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>梳理竞品在任务前、进行中、完成后和回访阶段展示的进度、成果、认可与下一步行动</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>调研中</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>首轮竞品：GitHub、Microsoft Learn、Trailhead、Stack Overflow、Kaggle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>T024</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>全站反馈与激励触点</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>交互</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>不同触点应提供与当前任务相关的反馈，避免把积分、徽章和排行榜集中堆叠</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>定义即时反馈、阶段反馈、成果证明、社会认可和再次行动的出现时机与跳转关系</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>调研中</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>待竞品分析后确认各页面的反馈强度与呈现方式</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2E53FA"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="37" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="37" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="31" customHeight="1">
+      <x:c r="A1" s="107" t="str">
+        <x:v>反馈与激励触点地图</x:v>
+      </x:c>
+      <x:c r="B1" s="107"/>
+      <x:c r="C1" s="107"/>
+      <x:c r="D1" s="107"/>
+      <x:c r="E1" s="107"/>
+      <x:c r="F1" s="107"/>
+      <x:c r="G1" s="107"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="109" t="str">
+        <x:v>按用户真实任务串联反馈：平台反馈什么、用什么证据证明、如何把用户推向下一步。首页只承接公共榜单摘要。</x:v>
+      </x:c>
+      <x:c r="B2" s="109"/>
+      <x:c r="C2" s="109"/>
+      <x:c r="D2" s="109"/>
+      <x:c r="E2" s="109"/>
+      <x:c r="F2" s="109"/>
+      <x:c r="G2" s="109"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="113" t="str">
+        <x:v>触点</x:v>
+      </x:c>
+      <x:c r="B4" s="113" t="str">
+        <x:v>用户阶段／场景</x:v>
+      </x:c>
+      <x:c r="C4" s="113" t="str">
+        <x:v>触发时机</x:v>
+      </x:c>
+      <x:c r="D4" s="113" t="str">
+        <x:v>平台反馈</x:v>
+      </x:c>
+      <x:c r="E4" s="113" t="str">
+        <x:v>可信证据</x:v>
+      </x:c>
+      <x:c r="F4" s="113" t="str">
+        <x:v>激励呈现</x:v>
+      </x:c>
+      <x:c r="G4" s="113" t="str">
+        <x:v>下一步行动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="72" customHeight="1">
+      <x:c r="A5" s="116" t="str">
+        <x:v>首页成长榜</x:v>
+      </x:c>
+      <x:c r="B5" s="116" t="str">
+        <x:v>发现榜样、判断自己是否值得参与</x:v>
+      </x:c>
+      <x:c r="C5" s="116" t="str">
+        <x:v>进入首页或切换榜单页签</x:v>
+      </x:c>
+      <x:c r="D5" s="116" t="str">
+        <x:v>呈现学习成长、实战突破、社区共建三类代表行为</x:v>
+      </x:c>
+      <x:c r="E5" s="116" t="str">
+        <x:v>阶段、任务成果、验证标签、采纳／复用证据</x:v>
+      </x:c>
+      <x:c r="F5" s="116" t="str">
+        <x:v>同阶段＋本周公共榜单；轻量展示用户名和行为</x:v>
+      </x:c>
+      <x:c r="G5" s="116" t="str">
+        <x:v>进入完整榜单、案例详情或开始自己的任务</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="A6" s="115" t="str">
+        <x:v>AI学习方案</x:v>
+      </x:c>
+      <x:c r="B6" s="115" t="str">
+        <x:v>确认目标并开始适合自己的学习路径</x:v>
+      </x:c>
+      <x:c r="C6" s="115" t="str">
+        <x:v>完成目标追问、确认学习方案</x:v>
+      </x:c>
+      <x:c r="D6" s="115" t="str">
+        <x:v>解释为什么推荐这条路径，并显示当前起点</x:v>
+      </x:c>
+      <x:c r="E6" s="115" t="str">
+        <x:v>用户目标、基础、环境、已确认答案</x:v>
+      </x:c>
+      <x:c r="F6" s="115" t="str">
+        <x:v>路径确认反馈；不做积分排名</x:v>
+      </x:c>
+      <x:c r="G6" s="115" t="str">
+        <x:v>进入课程预览或修改方案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" s="116" t="str">
+        <x:v>课程／实验学习</x:v>
+      </x:c>
+      <x:c r="B7" s="116" t="str">
+        <x:v>掌握知识并完成验证</x:v>
+      </x:c>
+      <x:c r="C7" s="116" t="str">
+        <x:v>完成单元、测验或实验</x:v>
+      </x:c>
+      <x:c r="D7" s="116" t="str">
+        <x:v>告诉用户掌握了什么、哪里还不稳、是否达到实践条件</x:v>
+      </x:c>
+      <x:c r="E7" s="116" t="str">
+        <x:v>首次掌握知识点、测验结果、实验运行和验收</x:v>
+      </x:c>
+      <x:c r="F7" s="116" t="str">
+        <x:v>阶段徽章、能力节点、继续学习建议</x:v>
+      </x:c>
+      <x:c r="G7" s="116" t="str">
+        <x:v>进入下一单元、复习薄弱点或进入 IDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="115" t="str">
+        <x:v>IDE实践／调试</x:v>
+      </x:c>
+      <x:c r="B8" s="115" t="str">
+        <x:v>解决真实开发问题</x:v>
+      </x:c>
+      <x:c r="C8" s="115" t="str">
+        <x:v>运行代码、出现错误、完成修复</x:v>
+      </x:c>
+      <x:c r="D8" s="115" t="str">
+        <x:v>反馈错误根因、修复是否有效、性能或稳定性变化</x:v>
+      </x:c>
+      <x:c r="E8" s="115" t="str">
+        <x:v>可复现运行结果、错误码、前后对比、任务验收</x:v>
+      </x:c>
+      <x:c r="F8" s="115" t="str">
+        <x:v>实战成果记录；可进入实战突破榜</x:v>
+      </x:c>
+      <x:c r="G8" s="115" t="str">
+        <x:v>保存为实践成果、继续优化或提交案例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" s="116" t="str">
+        <x:v>社区反馈／抓虫</x:v>
+      </x:c>
+      <x:c r="B9" s="116" t="str">
+        <x:v>纠正内容并改善他人的学习体验</x:v>
+      </x:c>
+      <x:c r="C9" s="116" t="str">
+        <x:v>提交问题、补充文档或修复建议</x:v>
+      </x:c>
+      <x:c r="D9" s="116" t="str">
+        <x:v>反馈审核、处理进度、是否采纳及影响范围</x:v>
+      </x:c>
+      <x:c r="E9" s="116" t="str">
+        <x:v>去重、审核、官方采纳、被引用或复用</x:v>
+      </x:c>
+      <x:c r="F9" s="116" t="str">
+        <x:v>社区共建榜、贡献徽章、案例署名</x:v>
+      </x:c>
+      <x:c r="G9" s="116" t="str">
+        <x:v>补充证据、查看处理结果或贡献下一条知识</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="115" t="str">
+        <x:v>个人空间／我的学习</x:v>
+      </x:c>
+      <x:c r="B10" s="115" t="str">
+        <x:v>回看长期成长并选择下一步</x:v>
+      </x:c>
+      <x:c r="C10" s="115" t="str">
+        <x:v>完成任务、获得认可或主动查看记录</x:v>
+      </x:c>
+      <x:c r="D10" s="115" t="str">
+        <x:v>汇总进度、能力、成果、贡献、历史荣誉和薄弱点</x:v>
+      </x:c>
+      <x:c r="E10" s="115" t="str">
+        <x:v>跨页面任务记录和验证结果</x:v>
+      </x:c>
+      <x:c r="F10" s="115" t="str">
+        <x:v>个人成长档案、徽章、历史排名</x:v>
+      </x:c>
+      <x:c r="G10" s="115" t="str">
+        <x:v>继续学习、复习、挑战更高难度或参与贡献</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="72" customHeight="1">
+      <x:c r="A11" s="116" t="str">
+        <x:v>AI智能学伴</x:v>
+      </x:c>
+      <x:c r="B11" s="116" t="str">
+        <x:v>理解反馈并把反馈转成行动</x:v>
+      </x:c>
+      <x:c r="C11" s="116" t="str">
+        <x:v>用户询问成长、遇到阻塞或完成阶段任务</x:v>
+      </x:c>
+      <x:c r="D11" s="116" t="str">
+        <x:v>解释成绩／成果来源，指出差距并给出下一步建议</x:v>
+      </x:c>
+      <x:c r="E11" s="116" t="str">
+        <x:v>读取当前页面上下文、个人记录和可信来源</x:v>
+      </x:c>
+      <x:c r="F11" s="116" t="str">
+        <x:v>个性化里程碑与行动建议；不单独制造刷榜指标</x:v>
+      </x:c>
+      <x:c r="G11" s="116" t="str">
+        <x:v>跳转到具体课程、实验、问题或社区任务</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2887,10 +3174,10 @@
         <x:v>切换榜单；查看完整榜单</x:v>
       </x:c>
       <x:c r="H15" s="51" t="str">
-        <x:v>具体信息结构和交互暂挂起</x:v>
+        <x:v>进入跨触点竞品分析与机制设计</x:v>
       </x:c>
       <x:c r="I15" s="51" t="str">
-        <x:v>保留产品机制定义；个人反馈进入我的学习或AI智能学伴</x:v>
+        <x:v>首页承接公共榜单摘要；个人反馈与行动激励需连接课程生成、学习、实践、社区、我的学习和AI学伴</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>